<commit_message>
2018-11-29 Sprawdzenie i uzupełnienie widoków dla modeli Szkoła, RokSzkolny, Uczeń, Klasa, klasyUcznia
</commit_message>
<xml_diff>
--- a/system.xlsx
+++ b/system.xlsx
@@ -4,10 +4,11 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12648" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
+    <sheet name="Arkusz2" sheetId="2" r:id="rId2"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Arkusz1!$A$1:$G$33</definedName>
@@ -22,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="88">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="90">
   <si>
     <t>szkoly</t>
   </si>
@@ -286,6 +287,12 @@
   </si>
   <si>
     <t>kolejność</t>
+  </si>
+  <si>
+    <t>Data</t>
+  </si>
+  <si>
+    <t>rozmiar folderu pomoc</t>
   </si>
 </sst>
 </file>
@@ -329,10 +336,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
@@ -1240,4 +1249,35 @@
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:B2"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="10.44140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>88</v>
+      </c>
+      <c r="B1" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A2" s="3">
+        <v>43432</v>
+      </c>
+      <c r="B2" s="4">
+        <v>4764294</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
2018-12-01 Utworzenie widoku uczniowieKlasy (wszyscy - dane uczniów) dla Klasy
</commit_message>
<xml_diff>
--- a/system.xlsx
+++ b/system.xlsx
@@ -299,7 +299,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -309,6 +309,13 @@
     </font>
     <font>
       <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -333,18 +340,21 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="2" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="3" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normalny" xfId="0" builtinId="0"/>
+    <cellStyle name="Procentowy" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1253,14 +1263,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:B2"/>
+  <dimension ref="A1:D6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="10.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
         <v>88</v>
       </c>
@@ -1268,12 +1278,76 @@
         <v>89</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A2" s="3">
-        <v>43432</v>
+        <v>43425</v>
       </c>
       <c r="B2" s="4">
-        <v>4764294</v>
+        <v>1157968</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A3" s="3">
+        <v>43426</v>
+      </c>
+      <c r="B3" s="4">
+        <v>1127528</v>
+      </c>
+      <c r="C3" s="5">
+        <f>B3/B2</f>
+        <v>0.97371257236814834</v>
+      </c>
+      <c r="D3" s="5">
+        <f>B3/$B$2</f>
+        <v>0.97371257236814834</v>
+      </c>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A4" s="3">
+        <v>43427</v>
+      </c>
+      <c r="B4" s="4">
+        <v>1124292</v>
+      </c>
+      <c r="C4" s="5">
+        <f t="shared" ref="C4:C6" si="0">B4/B3</f>
+        <v>0.99713000475376223</v>
+      </c>
+      <c r="D4" s="5">
+        <f t="shared" ref="D4:D6" si="1">B4/$B$2</f>
+        <v>0.97091802191424981</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A5" s="3">
+        <v>43428</v>
+      </c>
+      <c r="B5" s="4">
+        <v>1105197</v>
+      </c>
+      <c r="C5" s="5">
+        <f t="shared" si="0"/>
+        <v>0.98301597805552299</v>
+      </c>
+      <c r="D5" s="5">
+        <f t="shared" si="1"/>
+        <v>0.95442792892376993</v>
+      </c>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A6" s="3">
+        <v>43433</v>
+      </c>
+      <c r="B6" s="4">
+        <v>1031626</v>
+      </c>
+      <c r="C6" s="5">
+        <f t="shared" si="0"/>
+        <v>0.93343177732114724</v>
+      </c>
+      <c r="D6" s="5">
+        <f t="shared" si="1"/>
+        <v>0.89089335802025615</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
2018-12-01 Poprawienie wyświetlania widoków: wyświetlenie widoku table dla Uczniów, Klas i UczniaKlas dla Modeli Szkoła, RokSzkolny, Uczeń i Klasa
</commit_message>
<xml_diff>
--- a/system.xlsx
+++ b/system.xlsx
@@ -1263,7 +1263,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:D7"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
@@ -1310,11 +1310,11 @@
         <v>1124292</v>
       </c>
       <c r="C4" s="5">
-        <f t="shared" ref="C4:C6" si="0">B4/B3</f>
+        <f t="shared" ref="C4:C7" si="0">B4/B3</f>
         <v>0.99713000475376223</v>
       </c>
       <c r="D4" s="5">
-        <f t="shared" ref="D4:D6" si="1">B4/$B$2</f>
+        <f t="shared" ref="D4:D7" si="1">B4/$B$2</f>
         <v>0.97091802191424981</v>
       </c>
     </row>
@@ -1348,6 +1348,22 @@
       <c r="D6" s="5">
         <f t="shared" si="1"/>
         <v>0.89089335802025615</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A7" s="3">
+        <v>43435</v>
+      </c>
+      <c r="B7" s="4">
+        <v>1028308</v>
+      </c>
+      <c r="C7" s="5">
+        <f t="shared" si="0"/>
+        <v>0.99678371813040767</v>
+      </c>
+      <c r="D7" s="5">
+        <f t="shared" si="1"/>
+        <v>0.88802799386511544</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
2018-12-05 Dodanie możliwości sortowania klasUczniów dla widoku showStudents dla Klasy oraz showClasses dla Ucznia
</commit_message>
<xml_diff>
--- a/system.xlsx
+++ b/system.xlsx
@@ -1263,7 +1263,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D7"/>
+  <dimension ref="A1:D8"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
@@ -1310,11 +1310,11 @@
         <v>1124292</v>
       </c>
       <c r="C4" s="5">
-        <f t="shared" ref="C4:C7" si="0">B4/B3</f>
+        <f t="shared" ref="C4:C8" si="0">B4/B3</f>
         <v>0.99713000475376223</v>
       </c>
       <c r="D4" s="5">
-        <f t="shared" ref="D4:D7" si="1">B4/$B$2</f>
+        <f t="shared" ref="D4:D8" si="1">B4/$B$2</f>
         <v>0.97091802191424981</v>
       </c>
     </row>
@@ -1364,6 +1364,22 @@
       <c r="D7" s="5">
         <f t="shared" si="1"/>
         <v>0.88802799386511544</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A8" s="3">
+        <v>43438</v>
+      </c>
+      <c r="B8" s="4">
+        <v>1023132</v>
+      </c>
+      <c r="C8" s="5">
+        <f t="shared" si="0"/>
+        <v>0.99496648863959047</v>
+      </c>
+      <c r="D8" s="5">
+        <f t="shared" si="1"/>
+        <v>0.88355809486963366</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
2018-12-06 Poprawki w dodawaniu/modyfikowaniu dla modelu StudentClasses(klasy ucznia)
</commit_message>
<xml_diff>
--- a/system.xlsx
+++ b/system.xlsx
@@ -1263,7 +1263,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:D9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
@@ -1310,11 +1310,11 @@
         <v>1124292</v>
       </c>
       <c r="C4" s="5">
-        <f t="shared" ref="C4:C8" si="0">B4/B3</f>
+        <f t="shared" ref="C4:C9" si="0">B4/B3</f>
         <v>0.99713000475376223</v>
       </c>
       <c r="D4" s="5">
-        <f t="shared" ref="D4:D8" si="1">B4/$B$2</f>
+        <f t="shared" ref="D4:D9" si="1">B4/$B$2</f>
         <v>0.97091802191424981</v>
       </c>
     </row>
@@ -1380,6 +1380,22 @@
       <c r="D8" s="5">
         <f t="shared" si="1"/>
         <v>0.88355809486963366</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A9" s="3">
+        <v>43440</v>
+      </c>
+      <c r="B9" s="4">
+        <v>1020851</v>
+      </c>
+      <c r="C9" s="5">
+        <f t="shared" si="0"/>
+        <v>0.99777057114819989</v>
+      </c>
+      <c r="D9" s="5">
+        <f t="shared" si="1"/>
+        <v>0.88158826496068976</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
2018-12-14 Poprawki w konrolerze StudentClass
</commit_message>
<xml_diff>
--- a/system.xlsx
+++ b/system.xlsx
@@ -1263,7 +1263,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D10"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
@@ -1310,11 +1310,11 @@
         <v>1124292</v>
       </c>
       <c r="C4" s="5">
-        <f t="shared" ref="C4:C9" si="0">B4/B3</f>
+        <f t="shared" ref="C4:C10" si="0">B4/B3</f>
         <v>0.99713000475376223</v>
       </c>
       <c r="D4" s="5">
-        <f t="shared" ref="D4:D9" si="1">B4/$B$2</f>
+        <f t="shared" ref="D4:D10" si="1">B4/$B$2</f>
         <v>0.97091802191424981</v>
       </c>
     </row>
@@ -1396,6 +1396,22 @@
       <c r="D9" s="5">
         <f t="shared" si="1"/>
         <v>0.88158826496068976</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A10" s="3">
+        <v>43447</v>
+      </c>
+      <c r="B10" s="4">
+        <v>998445</v>
+      </c>
+      <c r="C10" s="5">
+        <f t="shared" si="0"/>
+        <v>0.97805164514703913</v>
+      </c>
+      <c r="D10" s="5">
+        <f t="shared" si="1"/>
+        <v>0.86223885288712643</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
2018-12-21 Dodanie sortowania ocen zadań oraz poprawki w wyświetlaniu widoku index dla wszystkich modeli
</commit_message>
<xml_diff>
--- a/system.xlsx
+++ b/system.xlsx
@@ -1263,7 +1263,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
@@ -1310,11 +1310,11 @@
         <v>1124292</v>
       </c>
       <c r="C4" s="5">
-        <f t="shared" ref="C4:C10" si="0">B4/B3</f>
+        <f t="shared" ref="C4:C11" si="0">B4/B3</f>
         <v>0.99713000475376223</v>
       </c>
       <c r="D4" s="5">
-        <f t="shared" ref="D4:D10" si="1">B4/$B$2</f>
+        <f t="shared" ref="D4:D11" si="1">B4/$B$2</f>
         <v>0.97091802191424981</v>
       </c>
     </row>
@@ -1412,6 +1412,22 @@
       <c r="D10" s="5">
         <f t="shared" si="1"/>
         <v>0.86223885288712643</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+      <c r="A11" s="3">
+        <v>43454</v>
+      </c>
+      <c r="B11" s="4">
+        <v>986032</v>
+      </c>
+      <c r="C11" s="5">
+        <f t="shared" si="0"/>
+        <v>0.98756766772330973</v>
+      </c>
+      <c r="D11" s="5">
+        <f t="shared" si="1"/>
+        <v>0.8515192129661614</v>
       </c>
     </row>
   </sheetData>

</xml_diff>